<commit_message>
chore: cross-cutting updates to vision/nature exports, knowledge base, project flow
Touched 31 files across:
- frontend: AnalysisCharts.tsx, Reports.tsx, Analysis.tsx, ProjectDetail.tsx,
  ProjectWizard.tsx, VisionAnalysis.tsx, App.tsx, GlobalPipelineProgress.tsx,
  analysisCharts/{ChartContext.ts, ModeAlert.tsx}, store/useAppStore.ts,
  types/index.ts, utils/exportBundle.ts
- backend services: clustering, design_engine, gemini_client, knowledge_base,
  nature_charts, project_context_builder, report_service, vision_client
- backend routes: analysis.py, nature_export.py, projects.py, vision.py
- backend models: analysis.py, project.py
- knowledge_base: Encoding_Dictionary.json, I_SVCs_Operations.json, SVCs_P_Evidence.json
- data: A_indicators.xlsx (binary, sha256-verified)

Built via safe pipeline (worktree -> /tmp -> hash-object). Every blob
size verified within (work_bytes - lines) <= blob <= work_bytes for text,
or exact byte+sha256 match for binary. No mid-token tails.
</commit_message>
<xml_diff>
--- a/packages/backend/data/A_indicators.xlsx
+++ b/packages/backend/data/A_indicators.xlsx
@@ -568,7 +568,6 @@
           <t>AI_g = \sum | (P_{gi} / \sum P_{g}) - (1/n) | / 2</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>%</t>
@@ -632,7 +631,6 @@
           <t>ASV (ASVI) = (Pixel_wall + Pixel_building + Pixel_fence + Pixel_skyscraper + Pixel_bench + Pixel_streetlight) / Pixel_total</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>%</t>
@@ -696,7 +694,6 @@
           <t>SV = 1.04165 + 2.00634 × WI + 0.49522 × C + 0.23200 × PR</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>%</t>
@@ -760,7 +757,6 @@
           <t>Brightness = (1/(3*M*N)) * sum_{b=1..3} sum_{i=0..N-1} sum_{j=0..M-1} I_bij</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>%</t>
@@ -824,7 +820,6 @@
           <t>L = mean of respondents' Likert ratings (1-5) for the test image relative to the benchmark image; aggregate across N respondents per image.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>%</t>
@@ -888,7 +883,6 @@
           <t>(Building Pixels / Total Pixels) * 100</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>%</t>
@@ -952,7 +946,6 @@
           <t>Pixel_Ceiling / Total_Pixels</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>%</t>
@@ -1016,7 +1009,6 @@
           <t>Compression Ratio = Size_compressed (JPEG) / Size_original (uncompressed)</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>%</t>
@@ -1080,7 +1072,6 @@
           <t>VE = -Sum_i (p_i * log(p_i)) (exact form per Qiu 2023 Supplementary Material SM I; main text only names the metric)</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>%</t>
@@ -1144,7 +1135,6 @@
           <t>CR = sum_{i=1..n} M * P_i * log(P_i) where M = sigma_rgyb + 0.3 * mu_rgyb; rg = R - G; yb = 0.5*(R + G) - B; sigma_rgyb = sqrt(sigma_rg^2 + sigma_yb^2</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>%</t>
@@ -1208,7 +1198,6 @@
           <t>CSI = sigma_rgyb + 0.3 * mu_rgyb</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>%</t>
@@ -1272,7 +1261,6 @@
           <t>Pixels_Dirt / Total_Pixels</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>%</t>
@@ -1336,7 +1324,6 @@
           <t>H = − Σ_{i=1}^{n} p_i · ln(p_i) / ln(n)</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>%</t>
@@ -1400,7 +1387,6 @@
           <t>M = 1 - ( (N - sqrt( sum_{i=1..5} n_i^2 )) / (N - sqrt(N)) )</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>%</t>
@@ -1464,7 +1450,6 @@
           <t>D = 1 - sum_i [n_i * (n_i - 1)] / [N * (N - 1)]</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>%</t>
@@ -1528,7 +1513,6 @@
           <t>Depth_mean = (1 / (M*N)) * sum_{i,j} D(i,j), where D(i,j) is the predicted depth value at pixel (i,j) of an MxN image</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>%</t>
@@ -1592,7 +1576,6 @@
           <t>EdgeDensity = N(edge pixels) / N(total pixels)</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>%</t>
@@ -1656,7 +1639,6 @@
           <t>1 - SVF_S, where SVF_S is the building-only sky view factor from simulation on a building height model (Li et al. 2018, building-only SVF formulation)</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>%</t>
@@ -1672,7 +1654,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>future_development</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1702,6 @@
           <t>DIE_i = [ (1/n)Sum_{k=1..n} B_k + (1/n)Sum_{k=1..n} T_k + (1/n)Sum_{k=1..n} W2_k ] / [ (1/n)Sum_{k=1..n} P1_k + (1/n)Sum_{k=1..n} F_k + (1/n)Sum_{k=1.</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>%</t>
@@ -1784,7 +1765,6 @@
           <t>Enclosure_trees = SVF_S − SVF_P, equivalently (1 − SVF_P) − (1 − SVF_S), where SVF_P is the GSV-based all-inclusive sky view factor and SVF_S is the s</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>%</t>
@@ -1800,7 +1780,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>future_development</t>
         </is>
       </c>
     </row>
@@ -1848,7 +1828,6 @@
           <t>ExG = 2*G - R - B ; per-image vegetation visibility = #{pixels: ExG &gt; Otsu(ExG)} / Pixels_total</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
           <t>%</t>
@@ -1912,7 +1891,6 @@
           <t>Category: Sealed vs Open/Railing</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>%</t>
@@ -1976,7 +1954,6 @@
           <t>S_ADI = (SDi - SDj) / SDi ; SDi = sqrt((1/N)*sum_i(Ai - mu_i)^2) ; SDj = sqrt((1/N)*sum_{i!=max}(Ai - mu_w)^2)</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
           <t>%</t>
@@ -2040,7 +2017,6 @@
           <t>S_API = sqrt( (1/N) * Sum_{i=1..N} (P_i - mu)^2 )</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>%</t>
@@ -2104,7 +2080,6 @@
           <t>P_ECI = sqrt( (1/N) * sum_j (CV_j - mu_CV)^2 ) / mu_CV ; CV_j = sqrt((1/Mj)*sum_i(Cij - mu_j)^2) / mu_j ; Cij = |idx_i - idx_{i+1}|</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t>%</t>
@@ -2168,7 +2143,6 @@
           <t>P_LN = sum_{i=1..N} Unique(Di)</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
           <t>%</t>
@@ -2232,7 +2206,6 @@
           <t>P_LV = max_{i in Foreground} Di</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
           <t>%</t>
@@ -2296,7 +2269,6 @@
           <t>S_ECI = Pb / (Py + Pb)</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
           <t>%</t>
@@ -2360,7 +2332,6 @@
           <t>S_ERI = 0.25 * P / sqrt(A)</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
           <t>%</t>
@@ -2424,7 +2395,6 @@
           <t>S_PSI = sqrt( (1/N) * sum_i ( (0.25*Pi/sqrt(Ai)) - mu )^2 ) / mu , where mu = (1/N) sum_i (0.25*Pi/sqrt(Ai))</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
           <t>%</t>
@@ -2488,7 +2458,6 @@
           <t>Pixels_Fence / Pixels_Visible (与其它 VI 元素一致,论文以 0–1 比值表达,可乘 100 得百分比)</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
           <t>%</t>
@@ -2552,7 +2521,6 @@
           <t>Db = lim (r-&gt;0) [log N(r) / log (1/r)]</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
           <t>%</t>
@@ -2616,7 +2584,6 @@
           <t>FreeSpace = (Pixels_grass + Pixels_earth + Pixels_ground + Pixels_outdoor_floor) / Pixels_total</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
           <t>%</t>
@@ -2680,7 +2647,6 @@
           <t>Step1: S_c = sum_k p_{c,k} over all images k for category c; Step2: sort p_{c,k} ascending; Step3: q_{c,k} = p_{c,k} / S_c; Step4: G_c = cumulative su</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>%</t>
@@ -2744,7 +2710,6 @@
           <t>vis_texture = - Σ_{i=0..255} Σ_{j=0..255} pg_{ij} * log2 C_{ij}  where C_{ij} is the normalized GLCM entry at offset (Δx, Δy)</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
           <t>%</t>
@@ -2808,7 +2773,6 @@
           <t>GCR = Pixel_groundcover / Pixel_total</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>%</t>
@@ -2872,7 +2836,6 @@
           <t>Contrast = Sum_{i=0}^{N-1} Sum_{j=0}^{N-1} (i - j)^2 * P(i, j)</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
           <t>%</t>
@@ -2936,7 +2899,6 @@
           <t>(Sum(Green_Pixels) / Sum(Total_Pixels)) * 100</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
           <t>%</t>
@@ -3000,7 +2962,6 @@
           <t>GVI_above = N(green_pixels with row &lt; horizon_row) / N(total_pixels);    horizon_row = (H_img / 2) - f_px * tan(pitch_rad);    Place Pulse 1.0 specifi</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
           <t>%</t>
@@ -3064,7 +3025,6 @@
           <t>GVI_below = N(green pixels with row &gt;= horizon_row) / N(total pixels); horizon_row = (H_image / 2) + f_px · tan(pitch_rad)  [Li et al. 2015, Eq. 4: Ho</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
           <t>%</t>
@@ -3128,7 +3088,6 @@
           <t>GV_band(k) = N(vegetation pixels in latitude band k) / N(total sky-map pixels in latitude band k), for k in {(0,22.5], (22.5,45], (45,67.5], (67.5,90]</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
           <t>%</t>
@@ -3192,7 +3151,6 @@
           <t>StdDev(GVI_front, GVI_back, GVI_left, GVI_right)</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>%</t>
@@ -3256,7 +3214,6 @@
           <t>Weighted Sum(Greenness, Openness, Enclosure, Walkability, Imageability)</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr">
         <is>
           <t>%</t>
@@ -3320,7 +3277,6 @@
           <t>I_k = (1/n) * sum_{j=1..n} B_jk + (1/n) * sum_{j=1..n} TL_jk + (1/n) * sum_{j=1..n} TS_jk</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr">
         <is>
           <t>%</t>
@@ -3384,7 +3340,6 @@
           <t>(1/3) * Sum_{b=1..3} sqrt( (1/(M*N)) * Sum_{i,j} (I_bij - I_b_bar)^2 )  where I_b_bar = (1/(M*N)) * Sum I_bij</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr">
         <is>
           <t>%</t>
@@ -3448,7 +3403,6 @@
           <t>IRI = N_categories_detected / N_categories_total</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
           <t>%</t>
@@ -3512,7 +3466,6 @@
           <t>Softmax probability vector output</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr">
         <is>
           <t>%</t>
@@ -3576,7 +3529,6 @@
           <t>MD = (P_road + P_car + P_bus + P_truck + P_freight_vehicle + P_small_motor_vehicle + P_railway) / P_all</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr">
         <is>
           <t>%</t>
@@ -3640,7 +3592,6 @@
           <t>Naturalness = arctan( Sum_{c in NaturalSet} A_c / Sum_{c in GreySet} A_c )</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr">
         <is>
           <t>%</t>
@@ -3704,7 +3655,6 @@
           <t>Ni = [ (1/n) Sum(Tn) + (1/n) Sum(Gn) + (1/n) Sum(W1n) + (1/n) Sum(M1n) + (1/n) Sum(P1n) ] / [ (1/n) Sum(Bn) + (1/n) Sum(W2n) + (1/n) Sum(Rn) + (1/n) S</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
           <t>%</t>
@@ -3768,7 +3718,6 @@
           <t>Ni = [(1/n) sum_{i=1..n} (Tn + Gn + W1n + M1n + P1n)] / [(1/n) sum_{i=1..n} (Bn + W2n + Rn + P2n + Fn)]</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>%</t>
@@ -3832,7 +3781,6 @@
           <t>NVGI = G0 / sqrt(R0 * B0)  where  R0 = (R_pixel - R_min)/(R_max - R_min), G0 = (G_pixel - G_min)/(G_max - G_min), B0 = (B_pixel - B_min)/(B_max - B_mi</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
           <t>%</t>
@@ -3896,7 +3844,6 @@
           <t>Overhead = (Pixels_tree + Pixels_ceiling + Pixels_canopy) / Pixels_total_topview</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
           <t>%</t>
@@ -3912,7 +3859,7 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>future_development</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3907,6 @@
           <t>PCI = (P_chair + P_toilet + P_bench + P_stool + P_trashcan + P_table + P_armchair + P_light + P_streetlight + P_bulletinboard) / P_all</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
           <t>%</t>
@@ -4024,7 +3970,6 @@
           <t>C = Sum_{i=1..n} M * Pi * log(Pi),  with rg = R - G;  yb = 0.5*(R+G) - B;  sigma_rgyb = sqrt(sigma_rg^2 + sigma_yb^2);  mu_rgyb = sqrt(mu_rg^2 + mu_yb</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
           <t>%</t>
@@ -4088,7 +4033,6 @@
           <t>Count of instances identified as 'peoples' using Mask R-CNN</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
           <t>%</t>
@@ -4152,7 +4096,6 @@
           <t>Level Diversity (richness) = N;  Level Diversity (entropy) = -Sum_{i=1..N} Pi * log2(Pi);  Level Diversity (simpson) = 1 - Sum_{i=1..N} (Pi/P)^2,  whe</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>%</t>
@@ -4216,7 +4159,6 @@
           <t>Pixels_Rider / Total_Pixels</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>%</t>
@@ -4280,7 +4222,6 @@
           <t>Pixel_road / Pixel_total</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr">
         <is>
           <t>%</t>
@@ -4344,7 +4285,6 @@
           <t>OtherFacilitiesRatio = Pixel_OtherFacilities / Total_Pixels (single aggregated class, not a sum of six sub-classes).</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr">
         <is>
           <t>%</t>
@@ -4408,7 +4348,6 @@
           <t>SFI = Wn / Rn</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr">
         <is>
           <t>%</t>
@@ -4472,7 +4411,6 @@
           <t>Per-point: shaded = 1 if sun position overlaps non-sky elements in the segmented fisheye skydome, else 0 (sunlit). Aggregated sunlit ratio: SunlitRati</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr">
         <is>
           <t>%</t>
@@ -4488,7 +4426,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>future_development</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4474,6 @@
           <t>Pixel_shrub / Pixel_total</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr">
         <is>
           <t>%</t>
@@ -4600,7 +4537,6 @@
           <t>SPD = P_road + P_path + P_wall + P_stair + P_pillar, where P_x = pixels_x / total_pixels</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr">
         <is>
           <t>%</t>
@@ -4664,7 +4600,6 @@
           <t>SQI = 1.507*GVI + 0.692*SVI + 0.447*EVI - 2.412*MVI - 0.011*SFI - 0.800*PCI - 0.060*VII + 1.414*ITI - 0.167*CCI + 0.208*SWI + 7.798*VEI - 6.344*IRI</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
           <t>%</t>
@@ -4728,7 +4663,6 @@
           <t>SSVF = Pixels_sign_symbol / Pixels_total</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr">
         <is>
           <t>%</t>
@@ -4792,7 +4726,6 @@
           <t>SVF = (∑_{i=0}^{n} ω · sky(i) / ∑_{i=0}^{n} ω) * 100%</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr">
         <is>
           <t>%</t>
@@ -4856,7 +4789,6 @@
           <t>|SVF_t - SVF_{t-1}|</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
           <t>%</t>
@@ -4872,7 +4804,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>future_development</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4852,6 @@
           <t>SVFdiff = SVFS - SVFP</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
           <t>%</t>
@@ -4936,7 +4867,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>future_development</t>
         </is>
       </c>
     </row>
@@ -4984,7 +4915,6 @@
           <t>Terrain_Ratio = N(pixels classified as 'terrain' by SegFormer/Cityscapes) / N(total pixels)</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr">
         <is>
           <t>%</t>
@@ -5048,7 +4978,6 @@
           <t>TR = (P_traffic_signal + P_sidewalk + P_railway) / P_all</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr">
         <is>
           <t>%</t>
@@ -5112,7 +5041,6 @@
           <t>TVF = Areat / Areas</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr">
         <is>
           <t>%</t>
@@ -5176,7 +5104,6 @@
           <t>(Simple) Pixels(Tree) / Total_Pixels  ;  (Hemispherical, Cai et al. 2023) Σ cos(Alti) · Ai · δi,green / Adome,cos</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr">
         <is>
           <t>%</t>
@@ -5240,7 +5167,6 @@
           <t>K-means Clustering(Gi, Si, Di, Ni)</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
       <c r="K75" t="inlineStr">
         <is>
           <t>%</t>
@@ -5304,7 +5230,6 @@
           <t>Sum(x_perc for x in {sidewalk, escalator, path, stairs, stairway, streetlight, bench, step})</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr">
         <is>
           <t>%</t>
@@ -5368,7 +5293,6 @@
           <t>1 - ((Tn/GVIn)^2 + (Pn/GVIn)^2 + (Gn/GVIn)^2)</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr">
         <is>
           <t>%</t>
@@ -5432,7 +5356,6 @@
           <t>(Pixels_car + Pixels_truck + Pixels_bus + Pixels_train + Pixels_motorcycle + Pixels_bicycle) / Total_pixels</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr">
         <is>
           <t>%</t>
@@ -5496,7 +5419,6 @@
           <t>VE = (Pixels_building + Pixels_wall + Pixels_tree + Pixels_fence) / Pixels_total · 100%   [exact element list to be confirmed against an authoritative</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr">
         <is>
           <t>%</t>
@@ -5560,7 +5482,6 @@
           <t>Spatialclustering_x = 0.5 * (SUM_i SUM_j x_i x_j) / xperc</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr">
         <is>
           <t>%</t>
@@ -5624,7 +5545,6 @@
           <t>v_x = GVI_E - GVI_W ; v_y = GVI_N - GVI_S ; |v| = sqrt(v_x^2 + v_y^2) ; theta = atan2(v_y, v_x)  [theta is implicit in the paper but standard]</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr">
         <is>
           <t>%</t>
@@ -5688,7 +5608,6 @@
           <t>VibrantGreen = N(pixels labelled vegetation AND HSV in healthy-green range) / N(total pixels)</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr">
         <is>
           <t>%</t>
@@ -5752,7 +5671,6 @@
           <t>VII = Pixels_motorised / Pixels_motorway</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr">
         <is>
           <t>%</t>
@@ -5816,7 +5734,6 @@
           <t>VQI = Sum_{k in {Safety, Lively, Beautiful, Wealthy, ...}} score_k   (verify against Wang/Ito/Biljecki 2024 Cities 104704)</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr">
         <is>
           <t>%</t>
@@ -5880,7 +5797,6 @@
           <t>Pn / (Pn + Rn)</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr">
         <is>
           <t>%</t>
@@ -5944,7 +5860,6 @@
           <t>VSD = - Sum_{i=1}^{N} p_i * ln(p_i), where p_i = C_i / C_veg</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr">
         <is>
           <t>%</t>
@@ -6008,7 +5923,6 @@
           <t>G_n = Σ_i ( G_i · L_i · D_i^α ) / Σ_i ( L_i · D_i^α )   [source: Ye, Xie, Fang, Jiang &amp; Wang 2019; cannot be verified against the supplied PDF for Lon</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr">
         <is>
           <t>%</t>
@@ -6024,7 +5938,7 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>future_development</t>
         </is>
       </c>
     </row>
@@ -6072,7 +5986,6 @@
           <t>Wall Ratio = Pixel_Wall / Total_Pixels</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr">
         <is>
           <t>%</t>
@@ -6136,7 +6049,6 @@
           <t>WVI = Pixels_water / Pixels_total</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
           <t>%</t>
@@ -6200,7 +6112,6 @@
           <t>arctan(flora / (grass + non_natural_elements))</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr">
         <is>
           <t>%</t>
@@ -6264,7 +6175,6 @@
           <t>W_i = ( (1/4) Σ_{j=1..4} P_j + (1/4) Σ_{j=1..4} F_j ) / ( (1/4) Σ_{j=1..4} Road_j )</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr">
         <is>
           <t>%</t>
@@ -6328,7 +6238,6 @@
           <t>VisualWalkability = (Sidewalk_pixels + Fence_pixels) / Road_pixels   (equivalently Pavement_pixels + Fence_pixels / Road_pixels under ADE20K-style lab</t>
         </is>
       </c>
-      <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr">
         <is>
           <t>%</t>
@@ -6372,7 +6281,6 @@
           <t>SceneRx Metrics Code 总览</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">

</xml_diff>